<commit_message>
fix(contest): update Shree Sanjay UK to 3/4 [1,1,1,0], revalidate 4/4 count to 42, and update canonical reports
</commit_message>
<xml_diff>
--- a/reports/Nandha_Engineering_College_Weekly_Contest_516_CSE_Cyber_Security_III_Year.xlsx
+++ b/reports/Nandha_Engineering_College_Weekly_Contest_516_CSE_Cyber_Security_III_Year.xlsx
@@ -1124,7 +1124,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>61</t>
         </is>
       </c>
     </row>
@@ -1240,10 +1240,10 @@
         </is>
       </c>
       <c r="B12" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" s="17" t="n">
         <v>13</v>
@@ -1264,7 +1264,7 @@
         <v>11</v>
       </c>
       <c r="J12" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1342,7 +1342,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -1554,10 +1554,10 @@
         <v>11</v>
       </c>
       <c r="J11" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
@@ -1864,10 +1864,10 @@
         <v>11</v>
       </c>
       <c r="J19" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1935,7 +1935,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -2206,12 +2206,12 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>SHREE SANJAY U K</t>
+          <t>AMRUTHA M</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>732224CCL03</t>
+          <t>732224CC002</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2229,15 +2229,15 @@
         <v>1</v>
       </c>
       <c r="H21" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" s="19" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="J21" s="19" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -2246,12 +2246,12 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>AMRUTHA M</t>
+          <t>BHARATH G</t>
         </is>
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>732224CC002</t>
+          <t>732224CC004</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
@@ -2286,12 +2286,12 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>BHARATH G</t>
+          <t>DHARUNRAJ K P</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>732224CC004</t>
+          <t>732224CC008</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2326,12 +2326,12 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>DHARUNRAJ K P</t>
+          <t>GOKUL P</t>
         </is>
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>732224CC008</t>
+          <t>732224CC010</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>GOKUL P</t>
+          <t>HARISH KUMAAR S</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>732224CC010</t>
+          <t>732224CC014</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2406,12 +2406,12 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>HARISH KUMAAR S</t>
+          <t>JANANI S</t>
         </is>
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>732224CC014</t>
+          <t>732224CC017</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
@@ -2446,12 +2446,12 @@
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>JANANI S</t>
+          <t>RAJESH R</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>732224CC017</t>
+          <t>732224CC039</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2486,12 +2486,12 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>RAJESH R</t>
+          <t>SARAN.R</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>732224CC039</t>
+          <t>732224CCL02</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
@@ -2526,12 +2526,12 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>SARAN.R</t>
+          <t>SHREE SANJAY U K</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>732224CCL02</t>
+          <t>732224CCL03</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -3152,7 +3152,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="G9" s="19" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10">
@@ -3336,7 +3336,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="C20" s="30" t="inlineStr">
         <is>
-          <t>94a47e67d366d22e1757b2ae77b691f59675b55b30e47fcbdda70706d832bde9</t>
+          <t>94c6d6eeefb395d95ef4c0a70598359d4f6ef0e639b9ee548c189ac04cb3fe6d</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5582,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -8216,7 +8216,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -11372,15 +11372,15 @@
         <v>1</v>
       </c>
       <c r="J69" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K69" s="22" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="L69" s="22" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="70">
@@ -11500,7 +11500,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -11573,12 +11573,12 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>732224CCL03</t>
+          <t>732224CC002</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>SHREE SANJAY U K</t>
+          <t>AMRUTHA M</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
@@ -11593,7 +11593,7 @@
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>shreesanjay</t>
+          <t>Amruthauma</t>
         </is>
       </c>
       <c r="G8" s="19" t="n">
@@ -11606,15 +11606,15 @@
         <v>1</v>
       </c>
       <c r="J8" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="23" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="L8" s="23" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -11623,12 +11623,12 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>732224CC002</t>
+          <t>732224CC004</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>AMRUTHA M</t>
+          <t>BHARATH G</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -11643,7 +11643,7 @@
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>Amruthauma</t>
+          <t>BHARATH1927</t>
         </is>
       </c>
       <c r="G9" s="19" t="n">
@@ -11673,12 +11673,12 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>732224CC004</t>
+          <t>732224CC008</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>BHARATH G</t>
+          <t>DHARUNRAJ K P</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>BHARATH1927</t>
+          <t>K_P_DHARUNRAJ</t>
         </is>
       </c>
       <c r="G10" s="19" t="n">
@@ -11723,12 +11723,12 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>732224CC008</t>
+          <t>732224CC010</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>DHARUNRAJ K P</t>
+          <t>GOKUL P</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>K_P_DHARUNRAJ</t>
+          <t>gokul_5405</t>
         </is>
       </c>
       <c r="G11" s="19" t="n">
@@ -11773,12 +11773,12 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>732224CC010</t>
+          <t>732224CC014</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>GOKUL P</t>
+          <t>HARISH KUMAAR S</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
@@ -11793,7 +11793,7 @@
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>gokul_5405</t>
+          <t>HarishVichu</t>
         </is>
       </c>
       <c r="G12" s="19" t="n">
@@ -11823,12 +11823,12 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>732224CC014</t>
+          <t>732224CC017</t>
         </is>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>HARISH KUMAAR S</t>
+          <t>JANANI S</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>HarishVichu</t>
+          <t>Jananii_26</t>
         </is>
       </c>
       <c r="G13" s="19" t="n">
@@ -11873,12 +11873,12 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>732224CC017</t>
+          <t>732224CC039</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>JANANI S</t>
+          <t>RAJESH R</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
@@ -11893,7 +11893,7 @@
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>Jananii_26</t>
+          <t>Rajesh1328</t>
         </is>
       </c>
       <c r="G14" s="19" t="n">
@@ -11923,12 +11923,12 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>732224CC039</t>
+          <t>732224CCL02</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>RAJESH R</t>
+          <t>SARAN.R</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>Rajesh1328</t>
+          <t>Saranraj_2580</t>
         </is>
       </c>
       <c r="G15" s="19" t="n">
@@ -11973,12 +11973,12 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>732224CCL02</t>
+          <t>732224CCL03</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>SARAN.R</t>
+          <t>SHREE SANJAY U K</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
@@ -11993,7 +11993,7 @@
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>Saranraj_2580</t>
+          <t>shreesanjay</t>
         </is>
       </c>
       <c r="G16" s="19" t="n">
@@ -12886,12 +12886,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -12927,14 +12927,14 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>WEEKLY CONTEST 516 — 4/4 PERFECT SOLVERS (1 STUDENTS)</t>
+          <t>WEEKLY CONTEST 516 — 4/4 PERFECT SOLVERS (0 STUDENTS)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -12999,56 +12999,6 @@
         <is>
           <t>Score</t>
         </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>732224CCL03</t>
-        </is>
-      </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>SHREE SANJAY U K</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>CSE(CS)</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>III</t>
-        </is>
-      </c>
-      <c r="F8" s="19" t="inlineStr">
-        <is>
-          <t>shreesanjay</t>
-        </is>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="23" t="inlineStr">
-        <is>
-          <t>4/4</t>
-        </is>
-      </c>
-      <c r="L8" s="23" t="n">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -13070,12 +13020,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -13111,14 +13061,14 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>WEEKLY CONTEST 516 — 3/4 SOLVERS (10 STUDENTS)</t>
+          <t>WEEKLY CONTEST 516 — 3/4 SOLVERS (11 STUDENTS)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -13591,12 +13541,12 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>732224CCL04</t>
+          <t>732224CCL03</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>SRIDHAR S</t>
+          <t>SHREE SANJAY U K</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
@@ -13611,7 +13561,7 @@
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>sridhar320076</t>
+          <t>shreesanjay</t>
         </is>
       </c>
       <c r="G16" s="19" t="n">
@@ -13641,47 +13591,97 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
+          <t>732224CCL04</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>SRIDHAR S</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>sridhar320076</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="23" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
           <t>732224CC059</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>YURJEEN J</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>CSE(CS)</t>
-        </is>
-      </c>
-      <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>III</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>CSE(CS)</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>Yurjeen26</t>
         </is>
       </c>
-      <c r="G17" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="23" t="inlineStr">
+      <c r="G18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="23" t="inlineStr">
         <is>
           <t>3/4</t>
         </is>
       </c>
-      <c r="L17" s="23" t="n">
+      <c r="L18" s="23" t="n">
         <v>12</v>
       </c>
     </row>
@@ -13752,7 +13752,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>
@@ -14536,7 +14536,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:10 AM IST</t>
+          <t>Contest Name: Weekly Contest 516   |   Session Date: 23.08.2026   |   Academic Year: 2026–2027   |   Institutional Roster Scope: 63 Students   |   Official Window: 08:00 AM – 09:30 AM IST   |   Generated At: 23 Aug 2026, 10:17 AM IST</t>
         </is>
       </c>
     </row>

</xml_diff>